<commit_message>
Update README to reflect version change to 2.1.0 and modify TPS latency test message
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish_chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD731F5-5BFD-4EB1-9C62-23496D16312D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44527807-D53D-4F1F-B0D2-005BA4128E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -36,11 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>v20.0/min</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>v2.0.0/avg</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -51,6 +47,29 @@
   </si>
   <si>
     <t>Message Count/tick</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>NaN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2.0.0/min</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2.1.0/min</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2.1.0/avg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>v2.1.0/max</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -435,138 +454,163 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="19.796875" customWidth="1"/>
     <col min="3" max="3" width="15.296875" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
     <col min="5" max="5" width="13.8984375" customWidth="1"/>
+    <col min="6" max="6" width="14.8984375" customWidth="1"/>
+    <col min="7" max="7" width="16.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A2">
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A3">
         <v>10</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>4</v>
       </c>
-      <c r="D2">
+      <c r="D3">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A4">
         <v>30</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>5</v>
       </c>
-      <c r="C3">
+      <c r="C4">
         <v>7</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A5">
         <v>50</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <v>6</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>9</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A5">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A6">
         <v>100</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>10</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>15</v>
       </c>
-      <c r="D5">
+      <c r="D6">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A6">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A7">
         <v>150</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>14</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>18</v>
       </c>
-      <c r="D6">
+      <c r="D7">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A8">
         <v>200</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <v>18</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>28</v>
       </c>
-      <c r="D7">
+      <c r="D8">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A8">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A9">
         <v>300</v>
       </c>
-      <c r="B8">
+      <c r="B9">
         <v>26</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>31</v>
       </c>
-      <c r="D8">
+      <c r="D9">
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A9">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A10">
         <v>378</v>
       </c>
-      <c r="B9">
+      <c r="B10">
         <v>33</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>38</v>
       </c>
-      <c r="D9">
+      <c r="D10">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latency image link in README: Change to version 2.2.0
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish_chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C733B7-236B-4A45-8CAC-58E6CEE188F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37CCEE1-18B7-46DA-B712-C918D88D441B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -72,6 +72,30 @@
   </si>
   <si>
     <t>1GB RAM and 250 char</t>
+  </si>
+  <si>
+    <t>50 min</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50 avg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50 max</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>250 max</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>250 avg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>250 min</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -455,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="19.796875" customWidth="1"/>
@@ -466,21 +490,30 @@
     <col min="7" max="7" width="16.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0</v>
       </c>
@@ -493,8 +526,17 @@
       <c r="D2">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>10</v>
       </c>
@@ -507,8 +549,17 @@
       <c r="D3">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>30</v>
       </c>
@@ -521,8 +572,17 @@
       <c r="D4">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>50</v>
       </c>
@@ -535,8 +595,17 @@
       <c r="D5">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>100</v>
       </c>
@@ -549,8 +618,17 @@
       <c r="D6">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>150</v>
       </c>
@@ -563,8 +641,17 @@
       <c r="D7">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>200</v>
       </c>
@@ -577,8 +664,17 @@
       <c r="D8">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+      <c r="G8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>250</v>
       </c>
@@ -591,8 +687,17 @@
       <c r="D9">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>300</v>
       </c>
@@ -605,8 +710,17 @@
       <c r="D10">
         <v>33</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>350</v>
       </c>
@@ -619,8 +733,17 @@
       <c r="D11">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>8</v>
+      </c>
+      <c r="G11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>400</v>
       </c>
@@ -632,6 +755,15 @@
       </c>
       <c r="D12">
         <v>47</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README for clarity and accuracy: Revise world type, benchmarking notes, and test message examples
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish_chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37CCEE1-18B7-46DA-B712-C918D88D441B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4F21BD-9387-4AEB-8E66-8ED97D2C6F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -86,15 +86,15 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>250 max</t>
+    <t>230 min</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>250 avg</t>
+    <t>230 avg</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>250 min</t>
+    <t>230 max</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -495,13 +495,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
         <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Increase maximum count limit from 500 to 1000 in EmbellishChatCommand; update feedback message accordingly
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish_chat\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4F21BD-9387-4AEB-8E66-8ED97D2C6F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25B700BE-BEF8-40DF-B809-5E8EB00B5B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId1"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId2"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId3"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId1"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId2"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId3"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -478,6 +479,301 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="21.296875" customWidth="1"/>
+    <col min="2" max="2" width="15.8984375" customWidth="1"/>
+    <col min="3" max="3" width="13.3984375" customWidth="1"/>
+    <col min="4" max="4" width="14.69921875" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="7" max="7" width="16.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>30</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>100</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>200</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>22</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A9">
+        <v>250</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>11</v>
+      </c>
+      <c r="D9">
+        <v>21</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A10">
+        <v>300</v>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>11</v>
+      </c>
+      <c r="D10">
+        <v>23</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>6</v>
+      </c>
+      <c r="G10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A11">
+        <v>350</v>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>12</v>
+      </c>
+      <c r="D11">
+        <v>23</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A12">
+        <v>400</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>13</v>
+      </c>
+      <c r="D12">
+        <v>22</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>7</v>
+      </c>
+      <c r="G12">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -772,7 +1068,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -931,7 +1227,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
docs(README): update version to 2.4.0 and adjust latency test parameters
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42F76800-906B-41D4-B29F-6B7311DEA94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358A2782-93D6-4CAF-8130-B4DAB8A09E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.3.0" sheetId="4" r:id="rId1"/>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId2"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId3"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId4"/>
+    <sheet name="v2.4.0" sheetId="5" r:id="rId1"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId2"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId3"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId4"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -96,6 +97,38 @@
   </si>
   <si>
     <t>230 max</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50/Plain Text</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50/Styling Only</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50/Mention Only</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50/Mixed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200/Plain Text</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200/Styling Only</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200/Mention Only</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200/Mixed</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -479,6 +512,260 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06116B37-F902-49E7-B259-88C657E3068D}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="19.09765625" customWidth="1"/>
+    <col min="2" max="2" width="15.19921875" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="22.09765625" customWidth="1"/>
+    <col min="6" max="6" width="20.3984375" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="23.09765625" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>100</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>8</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>200</v>
+      </c>
+      <c r="B5">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>10</v>
+      </c>
+      <c r="H5">
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>300</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
+        <v>12</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>22</v>
+      </c>
+      <c r="I6">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>400</v>
+      </c>
+      <c r="B7">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>11</v>
+      </c>
+      <c r="D7">
+        <v>12</v>
+      </c>
+      <c r="E7">
+        <v>12</v>
+      </c>
+      <c r="F7">
+        <v>11</v>
+      </c>
+      <c r="G7">
+        <v>17</v>
+      </c>
+      <c r="H7">
+        <v>27</v>
+      </c>
+      <c r="I7">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>500</v>
+      </c>
+      <c r="B8">
+        <v>8</v>
+      </c>
+      <c r="C8">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>14</v>
+      </c>
+      <c r="E8">
+        <v>16</v>
+      </c>
+      <c r="F8">
+        <v>12</v>
+      </c>
+      <c r="G8">
+        <v>19</v>
+      </c>
+      <c r="H8">
+        <v>33</v>
+      </c>
+      <c r="I8">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -773,7 +1060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1068,7 +1355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1227,7 +1514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
docs(README): refine TPS latency measurement description for clarity and accuracy
</commit_message>
<xml_diff>
--- a/docs/Latency per message.xlsx
+++ b/docs/Latency per message.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358A2782-93D6-4CAF-8130-B4DAB8A09E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C4F3986-D8F8-44D6-A70B-D38DECAFD9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -634,13 +634,13 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H4">
         <v>10</v>
       </c>
       <c r="I4">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.4">
@@ -663,13 +663,13 @@
         <v>8</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H5">
         <v>17</v>
       </c>
       <c r="I5">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.4">
@@ -692,7 +692,7 @@
         <v>10</v>
       </c>
       <c r="G6">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H6">
         <v>22</v>
@@ -721,13 +721,13 @@
         <v>11</v>
       </c>
       <c r="G7">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H7">
         <v>27</v>
       </c>
       <c r="I7">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.4">
@@ -750,13 +750,13 @@
         <v>12</v>
       </c>
       <c r="G8">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H8">
         <v>33</v>
       </c>
       <c r="I8">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>